<commit_message>
Auto sync Onetech 28/10/2026 18:06
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -76510,37 +76510,37 @@
         <v>45</v>
       </c>
       <c r="I579" s="3" t="s">
-        <v>972</v>
+        <v>1191</v>
       </c>
       <c r="J579" s="3" t="s">
-        <v>973</v>
+        <v>1192</v>
       </c>
       <c r="K579" s="3" t="s">
-        <v>974</v>
+        <v>1193</v>
       </c>
       <c r="L579" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M579" s="3" t="s">
-        <v>76</v>
+        <v>342</v>
       </c>
       <c r="N579" s="3" t="s">
-        <v>77</v>
+        <v>343</v>
       </c>
       <c r="O579" s="3" t="s">
-        <v>78</v>
+        <v>344</v>
       </c>
       <c r="P579" s="3" t="s">
-        <v>79</v>
+        <v>345</v>
       </c>
       <c r="Q579" s="5">
-        <v>4</v>
-      </c>
-      <c r="R579" s="3">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="R579" s="5">
+        <v>9</v>
       </c>
       <c r="S579" s="5">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="T579" s="3" t="s">
         <v>1172</v>
@@ -76563,8 +76563,8 @@
       <c r="Z579" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA579" s="7">
-        <v>430500</v>
+      <c r="AA579" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB579" s="7">
         <v>31</v>
@@ -76635,37 +76635,37 @@
         <v>45</v>
       </c>
       <c r="I580" s="3" t="s">
-        <v>1309</v>
+        <v>972</v>
       </c>
       <c r="J580" s="3" t="s">
-        <v>1000</v>
+        <v>973</v>
       </c>
       <c r="K580" s="3" t="s">
-        <v>1310</v>
+        <v>974</v>
       </c>
       <c r="L580" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M580" s="3" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="N580" s="3" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="O580" s="3" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="P580" s="3" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="Q580" s="5">
-        <v>16</v>
-      </c>
-      <c r="R580" s="5">
-        <v>16</v>
+        <v>4</v>
+      </c>
+      <c r="R580" s="3">
+        <v>0</v>
       </c>
       <c r="S580" s="5">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="T580" s="3" t="s">
         <v>1172</v>
@@ -76689,7 +76689,7 @@
         <v>46</v>
       </c>
       <c r="AA580" s="7">
-        <v>230000</v>
+        <v>430500</v>
       </c>
       <c r="AB580" s="7">
         <v>31</v>
@@ -76760,37 +76760,37 @@
         <v>45</v>
       </c>
       <c r="I581" s="3" t="s">
-        <v>993</v>
+        <v>1309</v>
       </c>
       <c r="J581" s="3" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="K581" s="3" t="s">
-        <v>995</v>
+        <v>1310</v>
       </c>
       <c r="L581" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M581" s="3" t="s">
-        <v>219</v>
+        <v>89</v>
       </c>
       <c r="N581" s="3" t="s">
-        <v>220</v>
+        <v>90</v>
       </c>
       <c r="O581" s="3" t="s">
-        <v>221</v>
+        <v>91</v>
       </c>
       <c r="P581" s="3" t="s">
-        <v>222</v>
+        <v>92</v>
       </c>
       <c r="Q581" s="5">
-        <v>6</v>
-      </c>
-      <c r="R581" s="3">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="R581" s="5">
+        <v>16</v>
       </c>
       <c r="S581" s="5">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="T581" s="3" t="s">
         <v>1172</v>
@@ -76814,7 +76814,7 @@
         <v>46</v>
       </c>
       <c r="AA581" s="7">
-        <v>728715</v>
+        <v>230000</v>
       </c>
       <c r="AB581" s="7">
         <v>31</v>
@@ -76885,37 +76885,37 @@
         <v>45</v>
       </c>
       <c r="I582" s="3" t="s">
-        <v>1311</v>
+        <v>993</v>
       </c>
       <c r="J582" s="3" t="s">
-        <v>1312</v>
+        <v>994</v>
       </c>
       <c r="K582" s="3" t="s">
-        <v>1313</v>
+        <v>995</v>
       </c>
       <c r="L582" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M582" s="3" t="s">
-        <v>183</v>
+        <v>219</v>
       </c>
       <c r="N582" s="3" t="s">
-        <v>184</v>
+        <v>220</v>
       </c>
       <c r="O582" s="3" t="s">
-        <v>185</v>
+        <v>221</v>
       </c>
       <c r="P582" s="3" t="s">
-        <v>186</v>
+        <v>222</v>
       </c>
       <c r="Q582" s="5">
-        <v>16</v>
-      </c>
-      <c r="R582" s="5">
-        <v>15</v>
+        <v>6</v>
+      </c>
+      <c r="R582" s="3">
+        <v>0</v>
       </c>
       <c r="S582" s="5">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="T582" s="3" t="s">
         <v>1172</v>
@@ -76939,7 +76939,7 @@
         <v>46</v>
       </c>
       <c r="AA582" s="7">
-        <v>765271</v>
+        <v>728715</v>
       </c>
       <c r="AB582" s="7">
         <v>31</v>
@@ -77010,13 +77010,13 @@
         <v>45</v>
       </c>
       <c r="I583" s="3" t="s">
-        <v>1314</v>
+        <v>1311</v>
       </c>
       <c r="J583" s="3" t="s">
-        <v>1315</v>
+        <v>1312</v>
       </c>
       <c r="K583" s="3" t="s">
-        <v>1316</v>
+        <v>1313</v>
       </c>
       <c r="L583" s="3" t="s">
         <v>50</v>
@@ -77034,13 +77034,13 @@
         <v>186</v>
       </c>
       <c r="Q583" s="5">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R583" s="5">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="S583" s="5">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T583" s="3" t="s">
         <v>1172</v>
@@ -77064,7 +77064,7 @@
         <v>46</v>
       </c>
       <c r="AA583" s="7">
-        <v>744487</v>
+        <v>765271</v>
       </c>
       <c r="AB583" s="7">
         <v>31</v>
@@ -77135,13 +77135,13 @@
         <v>45</v>
       </c>
       <c r="I584" s="3" t="s">
-        <v>1014</v>
+        <v>1314</v>
       </c>
       <c r="J584" s="3" t="s">
-        <v>403</v>
+        <v>1315</v>
       </c>
       <c r="K584" s="3" t="s">
-        <v>1015</v>
+        <v>1316</v>
       </c>
       <c r="L584" s="3" t="s">
         <v>50</v>
@@ -77189,7 +77189,7 @@
         <v>46</v>
       </c>
       <c r="AA584" s="7">
-        <v>156000</v>
+        <v>744487</v>
       </c>
       <c r="AB584" s="7">
         <v>31</v>
@@ -77260,37 +77260,37 @@
         <v>45</v>
       </c>
       <c r="I585" s="3" t="s">
-        <v>352</v>
+        <v>1014</v>
       </c>
       <c r="J585" s="3" t="s">
-        <v>353</v>
+        <v>403</v>
       </c>
       <c r="K585" s="3" t="s">
-        <v>354</v>
+        <v>1015</v>
       </c>
       <c r="L585" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M585" s="3" t="s">
-        <v>62</v>
+        <v>183</v>
       </c>
       <c r="N585" s="3" t="s">
-        <v>63</v>
+        <v>184</v>
       </c>
       <c r="O585" s="3" t="s">
-        <v>64</v>
+        <v>185</v>
       </c>
       <c r="P585" s="3" t="s">
-        <v>65</v>
+        <v>186</v>
       </c>
       <c r="Q585" s="5">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="R585" s="5">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="S585" s="5">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="T585" s="3" t="s">
         <v>1172</v>
@@ -77314,7 +77314,7 @@
         <v>46</v>
       </c>
       <c r="AA585" s="7">
-        <v>561438</v>
+        <v>156000</v>
       </c>
       <c r="AB585" s="7">
         <v>31</v>
@@ -77385,37 +77385,37 @@
         <v>45</v>
       </c>
       <c r="I586" s="3" t="s">
-        <v>1016</v>
+        <v>352</v>
       </c>
       <c r="J586" s="3" t="s">
-        <v>639</v>
+        <v>353</v>
       </c>
       <c r="K586" s="3" t="s">
-        <v>1017</v>
+        <v>354</v>
       </c>
       <c r="L586" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M586" s="3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N586" s="3" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="O586" s="3" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="P586" s="3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="Q586" s="5">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="R586" s="5">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="S586" s="5">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="T586" s="3" t="s">
         <v>1172</v>
@@ -77439,7 +77439,7 @@
         <v>46</v>
       </c>
       <c r="AA586" s="7">
-        <v>690000</v>
+        <v>561438</v>
       </c>
       <c r="AB586" s="7">
         <v>31</v>
@@ -77510,37 +77510,37 @@
         <v>45</v>
       </c>
       <c r="I587" s="3" t="s">
-        <v>1024</v>
+        <v>1016</v>
       </c>
       <c r="J587" s="3" t="s">
-        <v>1025</v>
+        <v>639</v>
       </c>
       <c r="K587" s="3" t="s">
-        <v>1026</v>
+        <v>1017</v>
       </c>
       <c r="L587" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M587" s="3" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="N587" s="3" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="O587" s="3" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="P587" s="3" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="Q587" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R587" s="5">
         <v>6</v>
       </c>
       <c r="S587" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T587" s="3" t="s">
         <v>1172</v>
@@ -77563,8 +77563,8 @@
       <c r="Z587" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA587" s="3" t="s">
-        <v>46</v>
+      <c r="AA587" s="7">
+        <v>690000</v>
       </c>
       <c r="AB587" s="7">
         <v>31</v>
@@ -77635,34 +77635,34 @@
         <v>45</v>
       </c>
       <c r="I588" s="3" t="s">
-        <v>520</v>
+        <v>1024</v>
       </c>
       <c r="J588" s="3" t="s">
-        <v>195</v>
+        <v>1025</v>
       </c>
       <c r="K588" s="3" t="s">
-        <v>521</v>
+        <v>1026</v>
       </c>
       <c r="L588" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M588" s="3" t="s">
-        <v>140</v>
+        <v>76</v>
       </c>
       <c r="N588" s="3" t="s">
-        <v>141</v>
+        <v>77</v>
       </c>
       <c r="O588" s="3" t="s">
-        <v>142</v>
+        <v>78</v>
       </c>
       <c r="P588" s="3" t="s">
-        <v>143</v>
+        <v>79</v>
       </c>
       <c r="Q588" s="5">
+        <v>7</v>
+      </c>
+      <c r="R588" s="5">
         <v>6</v>
-      </c>
-      <c r="R588" s="5">
-        <v>5</v>
       </c>
       <c r="S588" s="5">
         <v>7</v>
@@ -77688,8 +77688,8 @@
       <c r="Z588" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA588" s="7">
-        <v>88881</v>
+      <c r="AA588" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB588" s="7">
         <v>31</v>
@@ -77760,37 +77760,37 @@
         <v>45</v>
       </c>
       <c r="I589" s="3" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="J589" s="3" t="s">
-        <v>525</v>
+        <v>195</v>
       </c>
       <c r="K589" s="3" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="L589" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M589" s="3" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="N589" s="3" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="O589" s="3" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="P589" s="3" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="Q589" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R589" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S589" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T589" s="3" t="s">
         <v>1172</v>
@@ -77814,7 +77814,7 @@
         <v>46</v>
       </c>
       <c r="AA589" s="7">
-        <v>694460</v>
+        <v>88881</v>
       </c>
       <c r="AB589" s="7">
         <v>31</v>
@@ -77885,37 +77885,37 @@
         <v>45</v>
       </c>
       <c r="I590" s="3" t="s">
-        <v>1317</v>
+        <v>524</v>
       </c>
       <c r="J590" s="3" t="s">
-        <v>1318</v>
+        <v>525</v>
       </c>
       <c r="K590" s="3" t="s">
-        <v>1319</v>
+        <v>526</v>
       </c>
       <c r="L590" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M590" s="3" t="s">
-        <v>219</v>
+        <v>147</v>
       </c>
       <c r="N590" s="3" t="s">
-        <v>220</v>
+        <v>148</v>
       </c>
       <c r="O590" s="3" t="s">
-        <v>221</v>
+        <v>149</v>
       </c>
       <c r="P590" s="3" t="s">
-        <v>222</v>
+        <v>150</v>
       </c>
       <c r="Q590" s="5">
-        <v>5</v>
-      </c>
-      <c r="R590" s="3">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="R590" s="5">
+        <v>6</v>
       </c>
       <c r="S590" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="T590" s="3" t="s">
         <v>1172</v>
@@ -77939,7 +77939,7 @@
         <v>46</v>
       </c>
       <c r="AA590" s="7">
-        <v>935250</v>
+        <v>694460</v>
       </c>
       <c r="AB590" s="7">
         <v>31</v>
@@ -78010,37 +78010,37 @@
         <v>45</v>
       </c>
       <c r="I591" s="3" t="s">
-        <v>1320</v>
+        <v>1317</v>
       </c>
       <c r="J591" s="3" t="s">
-        <v>1321</v>
+        <v>1318</v>
       </c>
       <c r="K591" s="3" t="s">
-        <v>1322</v>
+        <v>1319</v>
       </c>
       <c r="L591" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M591" s="3" t="s">
-        <v>342</v>
+        <v>219</v>
       </c>
       <c r="N591" s="3" t="s">
-        <v>343</v>
+        <v>220</v>
       </c>
       <c r="O591" s="3" t="s">
-        <v>344</v>
+        <v>221</v>
       </c>
       <c r="P591" s="3" t="s">
-        <v>345</v>
+        <v>222</v>
       </c>
       <c r="Q591" s="5">
-        <v>8</v>
-      </c>
-      <c r="R591" s="5">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="R591" s="3">
+        <v>0</v>
       </c>
       <c r="S591" s="5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="T591" s="3" t="s">
         <v>1172</v>
@@ -78063,8 +78063,8 @@
       <c r="Z591" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA591" s="3" t="s">
-        <v>46</v>
+      <c r="AA591" s="7">
+        <v>935250</v>
       </c>
       <c r="AB591" s="7">
         <v>31</v>
@@ -78135,37 +78135,37 @@
         <v>45</v>
       </c>
       <c r="I592" s="3" t="s">
-        <v>588</v>
+        <v>1320</v>
       </c>
       <c r="J592" s="3" t="s">
-        <v>589</v>
+        <v>1321</v>
       </c>
       <c r="K592" s="3" t="s">
-        <v>590</v>
+        <v>1322</v>
       </c>
       <c r="L592" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M592" s="3" t="s">
-        <v>76</v>
+        <v>342</v>
       </c>
       <c r="N592" s="3" t="s">
-        <v>77</v>
+        <v>343</v>
       </c>
       <c r="O592" s="3" t="s">
-        <v>78</v>
+        <v>344</v>
       </c>
       <c r="P592" s="3" t="s">
-        <v>79</v>
+        <v>345</v>
       </c>
       <c r="Q592" s="5">
-        <v>2</v>
-      </c>
-      <c r="R592" s="3">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="R592" s="5">
+        <v>7</v>
       </c>
       <c r="S592" s="5">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="T592" s="3" t="s">
         <v>1172</v>
@@ -78260,37 +78260,37 @@
         <v>45</v>
       </c>
       <c r="I593" s="3" t="s">
-        <v>1200</v>
+        <v>588</v>
       </c>
       <c r="J593" s="3" t="s">
-        <v>1201</v>
+        <v>589</v>
       </c>
       <c r="K593" s="3" t="s">
-        <v>1202</v>
+        <v>590</v>
       </c>
       <c r="L593" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M593" s="3" t="s">
-        <v>183</v>
+        <v>76</v>
       </c>
       <c r="N593" s="3" t="s">
-        <v>184</v>
+        <v>77</v>
       </c>
       <c r="O593" s="3" t="s">
-        <v>185</v>
+        <v>78</v>
       </c>
       <c r="P593" s="3" t="s">
-        <v>186</v>
+        <v>79</v>
       </c>
       <c r="Q593" s="5">
-        <v>27</v>
-      </c>
-      <c r="R593" s="5">
-        <v>26</v>
+        <v>2</v>
+      </c>
+      <c r="R593" s="3">
+        <v>0</v>
       </c>
       <c r="S593" s="5">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="T593" s="3" t="s">
         <v>1172</v>
@@ -78385,37 +78385,37 @@
         <v>45</v>
       </c>
       <c r="I594" s="3" t="s">
-        <v>591</v>
+        <v>1200</v>
       </c>
       <c r="J594" s="3" t="s">
-        <v>592</v>
+        <v>1201</v>
       </c>
       <c r="K594" s="3" t="s">
-        <v>593</v>
+        <v>1202</v>
       </c>
       <c r="L594" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M594" s="3" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="N594" s="3" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="O594" s="3" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="P594" s="3" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="Q594" s="5">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="R594" s="5">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="S594" s="5">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T594" s="3" t="s">
         <v>1172</v>
@@ -78510,13 +78510,13 @@
         <v>45</v>
       </c>
       <c r="I595" s="3" t="s">
-        <v>1303</v>
+        <v>591</v>
       </c>
       <c r="J595" s="3" t="s">
-        <v>1304</v>
+        <v>592</v>
       </c>
       <c r="K595" s="3" t="s">
-        <v>1305</v>
+        <v>593</v>
       </c>
       <c r="L595" s="3" t="s">
         <v>50</v>
@@ -78537,7 +78537,7 @@
         <v>12</v>
       </c>
       <c r="R595" s="5">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S595" s="5">
         <v>12</v>
@@ -78635,37 +78635,37 @@
         <v>45</v>
       </c>
       <c r="I596" s="3" t="s">
-        <v>1323</v>
+        <v>1303</v>
       </c>
       <c r="J596" s="3" t="s">
-        <v>1324</v>
+        <v>1304</v>
       </c>
       <c r="K596" s="3" t="s">
-        <v>1325</v>
+        <v>1305</v>
       </c>
       <c r="L596" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M596" s="3" t="s">
-        <v>76</v>
+        <v>147</v>
       </c>
       <c r="N596" s="3" t="s">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="O596" s="3" t="s">
-        <v>78</v>
+        <v>149</v>
       </c>
       <c r="P596" s="3" t="s">
-        <v>79</v>
+        <v>150</v>
       </c>
       <c r="Q596" s="5">
-        <v>3</v>
-      </c>
-      <c r="R596" s="3">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="R596" s="5">
+        <v>11</v>
       </c>
       <c r="S596" s="5">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="T596" s="3" t="s">
         <v>1172</v>
@@ -78688,8 +78688,8 @@
       <c r="Z596" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA596" s="7">
-        <v>230000</v>
+      <c r="AA596" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB596" s="7">
         <v>31</v>
@@ -78760,37 +78760,37 @@
         <v>45</v>
       </c>
       <c r="I597" s="3" t="s">
-        <v>632</v>
+        <v>1323</v>
       </c>
       <c r="J597" s="3" t="s">
-        <v>633</v>
+        <v>1324</v>
       </c>
       <c r="K597" s="3" t="s">
-        <v>634</v>
+        <v>1325</v>
       </c>
       <c r="L597" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M597" s="3" t="s">
-        <v>140</v>
+        <v>76</v>
       </c>
       <c r="N597" s="3" t="s">
-        <v>141</v>
+        <v>77</v>
       </c>
       <c r="O597" s="3" t="s">
-        <v>142</v>
+        <v>78</v>
       </c>
       <c r="P597" s="3" t="s">
-        <v>143</v>
+        <v>79</v>
       </c>
       <c r="Q597" s="5">
-        <v>9</v>
-      </c>
-      <c r="R597" s="5">
         <v>3</v>
       </c>
+      <c r="R597" s="3">
+        <v>0</v>
+      </c>
       <c r="S597" s="5">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="T597" s="3" t="s">
         <v>1172</v>
@@ -78814,7 +78814,7 @@
         <v>46</v>
       </c>
       <c r="AA597" s="7">
-        <v>1170238</v>
+        <v>230000</v>
       </c>
       <c r="AB597" s="7">
         <v>31</v>
@@ -78885,13 +78885,13 @@
         <v>45</v>
       </c>
       <c r="I598" s="3" t="s">
-        <v>1223</v>
+        <v>632</v>
       </c>
       <c r="J598" s="3" t="s">
-        <v>1224</v>
+        <v>633</v>
       </c>
       <c r="K598" s="3" t="s">
-        <v>1225</v>
+        <v>634</v>
       </c>
       <c r="L598" s="3" t="s">
         <v>50</v>
@@ -78909,13 +78909,13 @@
         <v>143</v>
       </c>
       <c r="Q598" s="5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="R598" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S598" s="5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="T598" s="3" t="s">
         <v>1172</v>
@@ -78939,7 +78939,7 @@
         <v>46</v>
       </c>
       <c r="AA598" s="7">
-        <v>1033851</v>
+        <v>1170238</v>
       </c>
       <c r="AB598" s="7">
         <v>31</v>
@@ -79010,13 +79010,13 @@
         <v>45</v>
       </c>
       <c r="I599" s="3" t="s">
-        <v>635</v>
+        <v>1223</v>
       </c>
       <c r="J599" s="3" t="s">
-        <v>636</v>
+        <v>1224</v>
       </c>
       <c r="K599" s="3" t="s">
-        <v>637</v>
+        <v>1225</v>
       </c>
       <c r="L599" s="3" t="s">
         <v>50</v>
@@ -79034,13 +79034,13 @@
         <v>143</v>
       </c>
       <c r="Q599" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R599" s="5">
+        <v>5</v>
+      </c>
+      <c r="S599" s="5">
         <v>6</v>
-      </c>
-      <c r="S599" s="5">
-        <v>7</v>
       </c>
       <c r="T599" s="3" t="s">
         <v>1172</v>
@@ -79064,7 +79064,7 @@
         <v>46</v>
       </c>
       <c r="AA599" s="7">
-        <v>243297</v>
+        <v>1033851</v>
       </c>
       <c r="AB599" s="7">
         <v>31</v>
@@ -79135,37 +79135,37 @@
         <v>45</v>
       </c>
       <c r="I600" s="3" t="s">
-        <v>644</v>
+        <v>635</v>
       </c>
       <c r="J600" s="3" t="s">
-        <v>645</v>
+        <v>636</v>
       </c>
       <c r="K600" s="3" t="s">
-        <v>646</v>
+        <v>637</v>
       </c>
       <c r="L600" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M600" s="3" t="s">
-        <v>342</v>
+        <v>140</v>
       </c>
       <c r="N600" s="3" t="s">
-        <v>343</v>
+        <v>141</v>
       </c>
       <c r="O600" s="3" t="s">
-        <v>344</v>
+        <v>142</v>
       </c>
       <c r="P600" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="Q600" s="3">
-        <v>0</v>
-      </c>
-      <c r="R600" s="3">
-        <v>0</v>
+        <v>143</v>
+      </c>
+      <c r="Q600" s="5">
+        <v>7</v>
+      </c>
+      <c r="R600" s="5">
+        <v>6</v>
       </c>
       <c r="S600" s="5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="T600" s="3" t="s">
         <v>1172</v>
@@ -79189,7 +79189,7 @@
         <v>46</v>
       </c>
       <c r="AA600" s="7">
-        <v>225000</v>
+        <v>243297</v>
       </c>
       <c r="AB600" s="7">
         <v>31</v>
@@ -79260,37 +79260,37 @@
         <v>45</v>
       </c>
       <c r="I601" s="3" t="s">
-        <v>1292</v>
+        <v>644</v>
       </c>
       <c r="J601" s="3" t="s">
-        <v>1293</v>
+        <v>645</v>
       </c>
       <c r="K601" s="3" t="s">
-        <v>1294</v>
+        <v>646</v>
       </c>
       <c r="L601" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M601" s="3" t="s">
-        <v>183</v>
+        <v>342</v>
       </c>
       <c r="N601" s="3" t="s">
-        <v>184</v>
+        <v>343</v>
       </c>
       <c r="O601" s="3" t="s">
-        <v>185</v>
+        <v>344</v>
       </c>
       <c r="P601" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="Q601" s="5">
-        <v>28</v>
-      </c>
-      <c r="R601" s="5">
-        <v>28</v>
+        <v>345</v>
+      </c>
+      <c r="Q601" s="3">
+        <v>0</v>
+      </c>
+      <c r="R601" s="3">
+        <v>0</v>
       </c>
       <c r="S601" s="5">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="T601" s="3" t="s">
         <v>1172</v>
@@ -79314,7 +79314,7 @@
         <v>46</v>
       </c>
       <c r="AA601" s="7">
-        <v>690000</v>
+        <v>225000</v>
       </c>
       <c r="AB601" s="7">
         <v>31</v>
@@ -79385,37 +79385,37 @@
         <v>45</v>
       </c>
       <c r="I602" s="3" t="s">
-        <v>1081</v>
+        <v>1292</v>
       </c>
       <c r="J602" s="3" t="s">
-        <v>1082</v>
+        <v>1293</v>
       </c>
       <c r="K602" s="3" t="s">
-        <v>1083</v>
+        <v>1294</v>
       </c>
       <c r="L602" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M602" s="3" t="s">
-        <v>69</v>
+        <v>183</v>
       </c>
       <c r="N602" s="3" t="s">
-        <v>70</v>
+        <v>184</v>
       </c>
       <c r="O602" s="3" t="s">
-        <v>71</v>
+        <v>185</v>
       </c>
       <c r="P602" s="3" t="s">
-        <v>72</v>
+        <v>186</v>
       </c>
       <c r="Q602" s="5">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="R602" s="5">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="S602" s="5">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="T602" s="3" t="s">
         <v>1172</v>
@@ -79439,7 +79439,7 @@
         <v>46</v>
       </c>
       <c r="AA602" s="7">
-        <v>230000</v>
+        <v>690000</v>
       </c>
       <c r="AB602" s="7">
         <v>31</v>
@@ -79510,37 +79510,37 @@
         <v>45</v>
       </c>
       <c r="I603" s="3" t="s">
-        <v>655</v>
+        <v>1081</v>
       </c>
       <c r="J603" s="3" t="s">
-        <v>656</v>
+        <v>1082</v>
       </c>
       <c r="K603" s="3" t="s">
-        <v>657</v>
+        <v>1083</v>
       </c>
       <c r="L603" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M603" s="3" t="s">
-        <v>147</v>
+        <v>69</v>
       </c>
       <c r="N603" s="3" t="s">
-        <v>148</v>
+        <v>70</v>
       </c>
       <c r="O603" s="3" t="s">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="P603" s="3" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="Q603" s="5">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="R603" s="5">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="S603" s="5">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="T603" s="3" t="s">
         <v>1172</v>
@@ -79564,7 +79564,7 @@
         <v>46</v>
       </c>
       <c r="AA603" s="7">
-        <v>2933624</v>
+        <v>230000</v>
       </c>
       <c r="AB603" s="7">
         <v>31</v>
@@ -79635,13 +79635,13 @@
         <v>45</v>
       </c>
       <c r="I604" s="3" t="s">
-        <v>673</v>
+        <v>655</v>
       </c>
       <c r="J604" s="3" t="s">
-        <v>674</v>
+        <v>656</v>
       </c>
       <c r="K604" s="3" t="s">
-        <v>675</v>
+        <v>657</v>
       </c>
       <c r="L604" s="3" t="s">
         <v>50</v>
@@ -79659,13 +79659,13 @@
         <v>150</v>
       </c>
       <c r="Q604" s="5">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="R604" s="5">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="S604" s="5">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="T604" s="3" t="s">
         <v>1172</v>
@@ -79689,7 +79689,7 @@
         <v>46</v>
       </c>
       <c r="AA604" s="7">
-        <v>468000</v>
+        <v>2933624</v>
       </c>
       <c r="AB604" s="7">
         <v>31</v>
@@ -79760,37 +79760,37 @@
         <v>45</v>
       </c>
       <c r="I605" s="3" t="s">
-        <v>1326</v>
+        <v>673</v>
       </c>
       <c r="J605" s="3" t="s">
-        <v>1327</v>
+        <v>674</v>
       </c>
       <c r="K605" s="3" t="s">
-        <v>1328</v>
+        <v>675</v>
       </c>
       <c r="L605" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M605" s="3" t="s">
-        <v>183</v>
+        <v>147</v>
       </c>
       <c r="N605" s="3" t="s">
-        <v>184</v>
+        <v>148</v>
       </c>
       <c r="O605" s="3" t="s">
-        <v>185</v>
+        <v>149</v>
       </c>
       <c r="P605" s="3" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="Q605" s="5">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="R605" s="5">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="S605" s="5">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="T605" s="3" t="s">
         <v>1172</v>
@@ -79813,8 +79813,8 @@
       <c r="Z605" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA605" s="3" t="s">
-        <v>46</v>
+      <c r="AA605" s="7">
+        <v>468000</v>
       </c>
       <c r="AB605" s="7">
         <v>31</v>
@@ -79885,37 +79885,37 @@
         <v>45</v>
       </c>
       <c r="I606" s="3" t="s">
-        <v>1329</v>
+        <v>1326</v>
       </c>
       <c r="J606" s="3" t="s">
-        <v>580</v>
+        <v>1327</v>
       </c>
       <c r="K606" s="3" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="L606" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M606" s="3" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="N606" s="3" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="O606" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="P606" s="3" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="Q606" s="5">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="R606" s="5">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="S606" s="5">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="T606" s="3" t="s">
         <v>1172</v>
@@ -79938,8 +79938,8 @@
       <c r="Z606" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA606" s="7">
-        <v>1523616</v>
+      <c r="AA606" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB606" s="7">
         <v>31</v>
@@ -80010,37 +80010,37 @@
         <v>45</v>
       </c>
       <c r="I607" s="3" t="s">
-        <v>718</v>
+        <v>1329</v>
       </c>
       <c r="J607" s="3" t="s">
-        <v>719</v>
+        <v>580</v>
       </c>
       <c r="K607" s="3" t="s">
-        <v>720</v>
+        <v>1330</v>
       </c>
       <c r="L607" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M607" s="3" t="s">
-        <v>89</v>
+        <v>190</v>
       </c>
       <c r="N607" s="3" t="s">
-        <v>90</v>
+        <v>191</v>
       </c>
       <c r="O607" s="3" t="s">
-        <v>91</v>
+        <v>192</v>
       </c>
       <c r="P607" s="3" t="s">
-        <v>92</v>
+        <v>193</v>
       </c>
       <c r="Q607" s="5">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="R607" s="5">
         <v>6</v>
       </c>
       <c r="S607" s="5">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="T607" s="3" t="s">
         <v>1172</v>
@@ -80063,8 +80063,8 @@
       <c r="Z607" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA607" s="3" t="s">
-        <v>46</v>
+      <c r="AA607" s="7">
+        <v>1523616</v>
       </c>
       <c r="AB607" s="7">
         <v>31</v>
@@ -80135,37 +80135,37 @@
         <v>45</v>
       </c>
       <c r="I608" s="3" t="s">
-        <v>1229</v>
+        <v>718</v>
       </c>
       <c r="J608" s="3" t="s">
-        <v>1230</v>
+        <v>719</v>
       </c>
       <c r="K608" s="3" t="s">
-        <v>1231</v>
+        <v>720</v>
       </c>
       <c r="L608" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M608" s="3" t="s">
-        <v>183</v>
+        <v>89</v>
       </c>
       <c r="N608" s="3" t="s">
-        <v>184</v>
+        <v>90</v>
       </c>
       <c r="O608" s="3" t="s">
-        <v>185</v>
+        <v>91</v>
       </c>
       <c r="P608" s="3" t="s">
-        <v>186</v>
+        <v>92</v>
       </c>
       <c r="Q608" s="5">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="R608" s="5">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="S608" s="5">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="T608" s="3" t="s">
         <v>1172</v>
@@ -80188,8 +80188,8 @@
       <c r="Z608" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA608" s="7">
-        <v>3323238</v>
+      <c r="AA608" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB608" s="7">
         <v>31</v>
@@ -80260,37 +80260,37 @@
         <v>45</v>
       </c>
       <c r="I609" s="3" t="s">
-        <v>1331</v>
+        <v>1229</v>
       </c>
       <c r="J609" s="3" t="s">
-        <v>1332</v>
+        <v>1230</v>
       </c>
       <c r="K609" s="3" t="s">
-        <v>1333</v>
+        <v>1231</v>
       </c>
       <c r="L609" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M609" s="3" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="N609" s="3" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="O609" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="P609" s="3" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="Q609" s="5">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="R609" s="5">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="S609" s="5">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="T609" s="3" t="s">
         <v>1172</v>
@@ -80314,7 +80314,7 @@
         <v>46</v>
       </c>
       <c r="AA609" s="7">
-        <v>286618</v>
+        <v>3323238</v>
       </c>
       <c r="AB609" s="7">
         <v>31</v>
@@ -80385,37 +80385,37 @@
         <v>45</v>
       </c>
       <c r="I610" s="3" t="s">
-        <v>1334</v>
+        <v>1331</v>
       </c>
       <c r="J610" s="3" t="s">
-        <v>1335</v>
+        <v>1332</v>
       </c>
       <c r="K610" s="3" t="s">
-        <v>1336</v>
+        <v>1333</v>
       </c>
       <c r="L610" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M610" s="3" t="s">
-        <v>62</v>
+        <v>190</v>
       </c>
       <c r="N610" s="3" t="s">
-        <v>63</v>
+        <v>191</v>
       </c>
       <c r="O610" s="3" t="s">
-        <v>64</v>
+        <v>192</v>
       </c>
       <c r="P610" s="3" t="s">
-        <v>65</v>
+        <v>193</v>
       </c>
       <c r="Q610" s="5">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="R610" s="5">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="S610" s="5">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="T610" s="3" t="s">
         <v>1172</v>
@@ -80438,8 +80438,8 @@
       <c r="Z610" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA610" s="3" t="s">
-        <v>46</v>
+      <c r="AA610" s="7">
+        <v>286618</v>
       </c>
       <c r="AB610" s="7">
         <v>31</v>
@@ -80510,37 +80510,37 @@
         <v>45</v>
       </c>
       <c r="I611" s="3" t="s">
-        <v>1191</v>
+        <v>1334</v>
       </c>
       <c r="J611" s="3" t="s">
-        <v>1192</v>
+        <v>1335</v>
       </c>
       <c r="K611" s="3" t="s">
-        <v>1193</v>
+        <v>1336</v>
       </c>
       <c r="L611" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M611" s="3" t="s">
-        <v>342</v>
+        <v>62</v>
       </c>
       <c r="N611" s="3" t="s">
-        <v>343</v>
+        <v>63</v>
       </c>
       <c r="O611" s="3" t="s">
-        <v>344</v>
+        <v>64</v>
       </c>
       <c r="P611" s="3" t="s">
-        <v>345</v>
+        <v>65</v>
       </c>
       <c r="Q611" s="5">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="R611" s="5">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="S611" s="5">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="T611" s="3" t="s">
         <v>1172</v>

</xml_diff>

<commit_message>
Auto sync Onetech 28/10/2026 18:54
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -64534,13 +64534,13 @@
         <v>157</v>
       </c>
       <c r="Q483" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R483" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S483" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T483" s="3" t="s">
         <v>1172</v>
@@ -66284,13 +66284,13 @@
         <v>157</v>
       </c>
       <c r="Q497" s="5">
+        <v>27</v>
+      </c>
+      <c r="R497" s="5">
         <v>26</v>
       </c>
-      <c r="R497" s="5">
-        <v>25</v>
-      </c>
       <c r="S497" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T497" s="3" t="s">
         <v>1172</v>

</xml_diff>

<commit_message>
Auto sync Onetech 28/10/2026 19:09
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -73409,13 +73409,13 @@
         <v>186</v>
       </c>
       <c r="Q554" s="5">
+        <v>27</v>
+      </c>
+      <c r="R554" s="5">
         <v>26</v>
       </c>
-      <c r="R554" s="5">
-        <v>25</v>
-      </c>
       <c r="S554" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T554" s="3" t="s">
         <v>1172</v>
@@ -75534,13 +75534,13 @@
         <v>186</v>
       </c>
       <c r="Q571" s="5">
+        <v>25</v>
+      </c>
+      <c r="R571" s="5">
         <v>24</v>
       </c>
-      <c r="R571" s="5">
-        <v>23</v>
-      </c>
       <c r="S571" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T571" s="3" t="s">
         <v>1172</v>
@@ -80284,13 +80284,13 @@
         <v>186</v>
       </c>
       <c r="Q609" s="5">
+        <v>24</v>
+      </c>
+      <c r="R609" s="5">
         <v>23</v>
       </c>
-      <c r="R609" s="5">
-        <v>22</v>
-      </c>
       <c r="S609" s="5">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T609" s="3" t="s">
         <v>1172</v>

</xml_diff>

<commit_message>
Auto sync Onetech 30/10/2026 09:26
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -65764,13 +65764,13 @@
         <v>54</v>
       </c>
       <c r="Q492" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R492" s="5">
         <v>17</v>
       </c>
       <c r="S492" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T492" s="3" t="s">
         <v>1207</v>
@@ -66514,13 +66514,13 @@
         <v>164</v>
       </c>
       <c r="Q498" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R498" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S498" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T498" s="3" t="s">
         <v>1207</v>
@@ -68014,13 +68014,13 @@
         <v>164</v>
       </c>
       <c r="Q510" s="5">
+        <v>29</v>
+      </c>
+      <c r="R510" s="5">
         <v>28</v>
       </c>
-      <c r="R510" s="5">
-        <v>27</v>
-      </c>
       <c r="S510" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T510" s="3" t="s">
         <v>1207</v>
@@ -68139,13 +68139,13 @@
         <v>210</v>
       </c>
       <c r="Q511" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R511" s="3">
         <v>0</v>
       </c>
       <c r="S511" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T511" s="3" t="s">
         <v>1207</v>
@@ -75264,13 +75264,13 @@
         <v>54</v>
       </c>
       <c r="Q568" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R568" s="5">
         <v>2</v>
       </c>
       <c r="S568" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T568" s="3" t="s">
         <v>1207</v>

</xml_diff>

<commit_message>
Auto sync Onetech 30/10/2026 13:30
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20240" uniqueCount="1384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20234" uniqueCount="1384">
   <si>
     <t>DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH</t>
   </si>
@@ -3661,6 +3661,24 @@
     <t>Lầu 2 toà A1, Đại Học Quốc Tế</t>
   </si>
   <si>
+    <t>3057968</t>
+  </si>
+  <si>
+    <t>Anh Hùng ( Trái Cây )</t>
+  </si>
+  <si>
+    <t>71, Đình Phong Phú</t>
+  </si>
+  <si>
+    <t>2340641</t>
+  </si>
+  <si>
+    <t>Victor</t>
+  </si>
+  <si>
+    <t>89/1/9C, Đường 8</t>
+  </si>
+  <si>
     <t>5028</t>
   </si>
   <si>
@@ -3670,24 +3688,6 @@
     <t xml:space="preserve">108, Đường 4 Đại Học Nông Lâm </t>
   </si>
   <si>
-    <t>3057968</t>
-  </si>
-  <si>
-    <t>Anh Hùng ( Trái Cây )</t>
-  </si>
-  <si>
-    <t>71, Đình Phong Phú</t>
-  </si>
-  <si>
-    <t>2340641</t>
-  </si>
-  <si>
-    <t>Victor</t>
-  </si>
-  <si>
-    <t>89/1/9C, Đường 8</t>
-  </si>
-  <si>
     <t>1-6JP933U</t>
   </si>
   <si>
@@ -3787,6 +3787,24 @@
     <t>208/6B, Đường 138</t>
   </si>
   <si>
+    <t>999137208</t>
+  </si>
+  <si>
+    <t>Tạp Hoá Hai Quân</t>
+  </si>
+  <si>
+    <t>19-20, Chợ Tăng Nhơn Phú B</t>
+  </si>
+  <si>
+    <t>4415</t>
+  </si>
+  <si>
+    <t>Cô Liên</t>
+  </si>
+  <si>
+    <t>16, Đường 120</t>
+  </si>
+  <si>
     <t>4107</t>
   </si>
   <si>
@@ -3794,24 +3812,6 @@
   </si>
   <si>
     <t>26, Chợ Linh Xuân</t>
-  </si>
-  <si>
-    <t>4415</t>
-  </si>
-  <si>
-    <t>Cô Liên</t>
-  </si>
-  <si>
-    <t>16, Đường 120</t>
-  </si>
-  <si>
-    <t>999137208</t>
-  </si>
-  <si>
-    <t>Tạp Hoá Hai Quân</t>
-  </si>
-  <si>
-    <t>19-20, Chợ Tăng Nhơn Phú B</t>
   </si>
   <si>
     <t>Mức 3 - Kệ CTP</t>
@@ -31013,14 +31013,14 @@
       <c r="P214" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="Q214" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R214" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S214" s="3" t="s">
-        <v>46</v>
+      <c r="Q214" s="5">
+        <v>1</v>
+      </c>
+      <c r="R214" s="5">
+        <v>1</v>
+      </c>
+      <c r="S214" s="5">
+        <v>1</v>
       </c>
       <c r="T214" s="3" t="s">
         <v>46</v>
@@ -57513,14 +57513,14 @@
       <c r="P426" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="Q426" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R426" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S426" s="3" t="s">
-        <v>46</v>
+      <c r="Q426" s="5">
+        <v>1</v>
+      </c>
+      <c r="R426" s="3">
+        <v>0</v>
+      </c>
+      <c r="S426" s="5">
+        <v>1</v>
       </c>
       <c r="T426" s="3" t="s">
         <v>46</v>
@@ -64002,16 +64002,16 @@
         <v>50</v>
       </c>
       <c r="M478" s="3" t="s">
-        <v>114</v>
+        <v>193</v>
       </c>
       <c r="N478" s="3" t="s">
-        <v>115</v>
+        <v>194</v>
       </c>
       <c r="O478" s="3" t="s">
-        <v>116</v>
+        <v>195</v>
       </c>
       <c r="P478" s="3" t="s">
-        <v>117</v>
+        <v>196</v>
       </c>
       <c r="Q478" s="3" t="s">
         <v>46</v>
@@ -64044,7 +64044,7 @@
         <v>10</v>
       </c>
       <c r="AA478" s="7">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AB478" s="7">
         <v>1</v>
@@ -64074,7 +64074,7 @@
         <v>58</v>
       </c>
       <c r="AK478" s="6">
-        <v>46300.730373495375</v>
+        <v>46307.90555991898</v>
       </c>
       <c r="AL478" s="3" t="s">
         <v>46</v>
@@ -64086,7 +64086,7 @@
         <v>58</v>
       </c>
       <c r="AO478" s="6">
-        <v>46300.730373495375</v>
+        <v>46307.90555991898</v>
       </c>
     </row>
     <row r="479" spans="1:41" x14ac:dyDescent="0.25">
@@ -64169,10 +64169,10 @@
         <v>10</v>
       </c>
       <c r="AA479" s="7">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="AB479" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC479" s="3" t="s">
         <v>1208</v>
@@ -64190,7 +64190,7 @@
         <v>1212</v>
       </c>
       <c r="AH479" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI479" s="3">
         <v>0</v>
@@ -64199,7 +64199,7 @@
         <v>58</v>
       </c>
       <c r="AK479" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
       <c r="AL479" s="3" t="s">
         <v>46</v>
@@ -64211,7 +64211,7 @@
         <v>58</v>
       </c>
       <c r="AO479" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
     </row>
     <row r="480" spans="1:41" x14ac:dyDescent="0.25">
@@ -64240,28 +64240,28 @@
         <v>45</v>
       </c>
       <c r="I480" s="3" t="s">
-        <v>1222</v>
+        <v>233</v>
       </c>
       <c r="J480" s="3" t="s">
-        <v>1223</v>
+        <v>234</v>
       </c>
       <c r="K480" s="3" t="s">
-        <v>1224</v>
+        <v>235</v>
       </c>
       <c r="L480" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M480" s="3" t="s">
-        <v>193</v>
+        <v>154</v>
       </c>
       <c r="N480" s="3" t="s">
-        <v>194</v>
+        <v>155</v>
       </c>
       <c r="O480" s="3" t="s">
-        <v>195</v>
+        <v>156</v>
       </c>
       <c r="P480" s="3" t="s">
-        <v>196</v>
+        <v>157</v>
       </c>
       <c r="Q480" s="3" t="s">
         <v>46</v>
@@ -64294,10 +64294,10 @@
         <v>10</v>
       </c>
       <c r="AA480" s="7">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="AB480" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC480" s="3" t="s">
         <v>1208</v>
@@ -64315,7 +64315,7 @@
         <v>1212</v>
       </c>
       <c r="AH480" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI480" s="3">
         <v>0</v>
@@ -64365,28 +64365,28 @@
         <v>45</v>
       </c>
       <c r="I481" s="3" t="s">
-        <v>233</v>
+        <v>1222</v>
       </c>
       <c r="J481" s="3" t="s">
-        <v>234</v>
+        <v>1223</v>
       </c>
       <c r="K481" s="3" t="s">
-        <v>235</v>
+        <v>1224</v>
       </c>
       <c r="L481" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M481" s="3" t="s">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="N481" s="3" t="s">
-        <v>155</v>
+        <v>115</v>
       </c>
       <c r="O481" s="3" t="s">
-        <v>156</v>
+        <v>116</v>
       </c>
       <c r="P481" s="3" t="s">
-        <v>157</v>
+        <v>117</v>
       </c>
       <c r="Q481" s="3" t="s">
         <v>46</v>
@@ -64419,7 +64419,7 @@
         <v>10</v>
       </c>
       <c r="AA481" s="7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AB481" s="7">
         <v>1</v>
@@ -64449,7 +64449,7 @@
         <v>58</v>
       </c>
       <c r="AK481" s="6">
-        <v>46301.91933796296</v>
+        <v>46300.730373495375</v>
       </c>
       <c r="AL481" s="3" t="s">
         <v>46</v>
@@ -64461,7 +64461,7 @@
         <v>58</v>
       </c>
       <c r="AO481" s="6">
-        <v>46301.91933796296</v>
+        <v>46300.730373495375</v>
       </c>
     </row>
     <row r="482" spans="1:41" x14ac:dyDescent="0.25">
@@ -65014,13 +65014,13 @@
         <v>140</v>
       </c>
       <c r="Q486" s="5">
+        <v>12</v>
+      </c>
+      <c r="R486" s="5">
         <v>10</v>
       </c>
-      <c r="R486" s="5">
-        <v>8</v>
-      </c>
       <c r="S486" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="T486" s="3" t="s">
         <v>1207</v>
@@ -65889,13 +65889,13 @@
         <v>65</v>
       </c>
       <c r="Q493" s="5">
+        <v>20</v>
+      </c>
+      <c r="R493" s="5">
         <v>19</v>
       </c>
-      <c r="R493" s="5">
-        <v>18</v>
-      </c>
       <c r="S493" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T493" s="3" t="s">
         <v>1207</v>
@@ -66014,13 +66014,13 @@
         <v>164</v>
       </c>
       <c r="Q494" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R494" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S494" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T494" s="3" t="s">
         <v>1207</v>
@@ -66990,37 +66990,37 @@
         <v>1228</v>
       </c>
       <c r="I502" s="3" t="s">
-        <v>1258</v>
+        <v>1121</v>
       </c>
       <c r="J502" s="3" t="s">
-        <v>1259</v>
+        <v>1122</v>
       </c>
       <c r="K502" s="3" t="s">
-        <v>1260</v>
+        <v>1123</v>
       </c>
       <c r="L502" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M502" s="3" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="N502" s="3" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="O502" s="3" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="P502" s="3" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="Q502" s="5">
-        <v>4</v>
-      </c>
-      <c r="R502" s="3">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="R502" s="5">
+        <v>12</v>
       </c>
       <c r="S502" s="5">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="T502" s="3" t="s">
         <v>1207</v>
@@ -67044,7 +67044,7 @@
         <v>46</v>
       </c>
       <c r="AA502" s="7">
-        <v>5510425</v>
+        <v>9672464</v>
       </c>
       <c r="AB502" s="7">
         <v>31</v>
@@ -67115,37 +67115,37 @@
         <v>1228</v>
       </c>
       <c r="I503" s="3" t="s">
-        <v>641</v>
+        <v>1126</v>
       </c>
       <c r="J503" s="3" t="s">
-        <v>642</v>
+        <v>1127</v>
       </c>
       <c r="K503" s="3" t="s">
-        <v>643</v>
+        <v>1128</v>
       </c>
       <c r="L503" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M503" s="3" t="s">
-        <v>147</v>
+        <v>207</v>
       </c>
       <c r="N503" s="3" t="s">
-        <v>148</v>
+        <v>208</v>
       </c>
       <c r="O503" s="3" t="s">
-        <v>149</v>
+        <v>209</v>
       </c>
       <c r="P503" s="3" t="s">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="Q503" s="5">
-        <v>2</v>
-      </c>
-      <c r="R503" s="3">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="R503" s="5">
+        <v>3</v>
       </c>
       <c r="S503" s="5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T503" s="3" t="s">
         <v>1207</v>
@@ -67169,7 +67169,7 @@
         <v>46</v>
       </c>
       <c r="AA503" s="7">
-        <v>5098703</v>
+        <v>7413795</v>
       </c>
       <c r="AB503" s="7">
         <v>31</v>
@@ -67240,37 +67240,37 @@
         <v>1228</v>
       </c>
       <c r="I504" s="3" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="J504" s="3" t="s">
-        <v>1262</v>
+        <v>1259</v>
       </c>
       <c r="K504" s="3" t="s">
-        <v>1263</v>
+        <v>1260</v>
       </c>
       <c r="L504" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M504" s="3" t="s">
-        <v>161</v>
+        <v>193</v>
       </c>
       <c r="N504" s="3" t="s">
-        <v>162</v>
+        <v>194</v>
       </c>
       <c r="O504" s="3" t="s">
-        <v>163</v>
+        <v>195</v>
       </c>
       <c r="P504" s="3" t="s">
-        <v>164</v>
+        <v>196</v>
       </c>
       <c r="Q504" s="5">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="R504" s="5">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="S504" s="5">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="T504" s="3" t="s">
         <v>1207</v>
@@ -67294,7 +67294,7 @@
         <v>46</v>
       </c>
       <c r="AA504" s="7">
-        <v>1728143</v>
+        <v>6340940</v>
       </c>
       <c r="AB504" s="7">
         <v>31</v>
@@ -67365,37 +67365,37 @@
         <v>1228</v>
       </c>
       <c r="I505" s="3" t="s">
-        <v>1121</v>
+        <v>1261</v>
       </c>
       <c r="J505" s="3" t="s">
-        <v>1122</v>
+        <v>1262</v>
       </c>
       <c r="K505" s="3" t="s">
-        <v>1123</v>
+        <v>1263</v>
       </c>
       <c r="L505" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M505" s="3" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="N505" s="3" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="O505" s="3" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="P505" s="3" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="Q505" s="5">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="R505" s="5">
+        <v>6</v>
+      </c>
+      <c r="S505" s="5">
         <v>10</v>
-      </c>
-      <c r="S505" s="5">
-        <v>11</v>
       </c>
       <c r="T505" s="3" t="s">
         <v>1207</v>
@@ -67419,7 +67419,7 @@
         <v>46</v>
       </c>
       <c r="AA505" s="7">
-        <v>9672464</v>
+        <v>1728143</v>
       </c>
       <c r="AB505" s="7">
         <v>31</v>
@@ -67490,37 +67490,37 @@
         <v>1228</v>
       </c>
       <c r="I506" s="3" t="s">
-        <v>1126</v>
+        <v>641</v>
       </c>
       <c r="J506" s="3" t="s">
-        <v>1127</v>
+        <v>642</v>
       </c>
       <c r="K506" s="3" t="s">
-        <v>1128</v>
+        <v>643</v>
       </c>
       <c r="L506" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M506" s="3" t="s">
-        <v>207</v>
+        <v>147</v>
       </c>
       <c r="N506" s="3" t="s">
-        <v>208</v>
+        <v>148</v>
       </c>
       <c r="O506" s="3" t="s">
-        <v>209</v>
+        <v>149</v>
       </c>
       <c r="P506" s="3" t="s">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="Q506" s="5">
-        <v>5</v>
-      </c>
-      <c r="R506" s="5">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="R506" s="3">
+        <v>0</v>
       </c>
       <c r="S506" s="5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T506" s="3" t="s">
         <v>1207</v>
@@ -67544,7 +67544,7 @@
         <v>46</v>
       </c>
       <c r="AA506" s="7">
-        <v>7413795</v>
+        <v>5098703</v>
       </c>
       <c r="AB506" s="7">
         <v>31</v>
@@ -67627,25 +67627,25 @@
         <v>50</v>
       </c>
       <c r="M507" s="3" t="s">
-        <v>193</v>
+        <v>147</v>
       </c>
       <c r="N507" s="3" t="s">
-        <v>194</v>
+        <v>148</v>
       </c>
       <c r="O507" s="3" t="s">
-        <v>195</v>
+        <v>149</v>
       </c>
       <c r="P507" s="3" t="s">
-        <v>196</v>
+        <v>150</v>
       </c>
       <c r="Q507" s="5">
-        <v>24</v>
-      </c>
-      <c r="R507" s="5">
-        <v>23</v>
+        <v>4</v>
+      </c>
+      <c r="R507" s="3">
+        <v>0</v>
       </c>
       <c r="S507" s="5">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="T507" s="3" t="s">
         <v>1207</v>
@@ -67669,7 +67669,7 @@
         <v>46</v>
       </c>
       <c r="AA507" s="7">
-        <v>6340940</v>
+        <v>5510425</v>
       </c>
       <c r="AB507" s="7">
         <v>31</v>
@@ -68764,13 +68764,13 @@
         <v>140</v>
       </c>
       <c r="Q516" s="5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="R516" s="5">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="S516" s="5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="T516" s="3" t="s">
         <v>1207</v>
@@ -74764,13 +74764,13 @@
         <v>196</v>
       </c>
       <c r="Q564" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R564" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S564" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T564" s="3" t="s">
         <v>1207</v>
@@ -74889,13 +74889,13 @@
         <v>140</v>
       </c>
       <c r="Q565" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R565" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S565" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="T565" s="3" t="s">
         <v>1207</v>
@@ -75115,13 +75115,13 @@
         <v>45</v>
       </c>
       <c r="I567" s="3" t="s">
-        <v>1264</v>
+        <v>1258</v>
       </c>
       <c r="J567" s="3" t="s">
-        <v>1265</v>
+        <v>1259</v>
       </c>
       <c r="K567" s="3" t="s">
-        <v>1266</v>
+        <v>1260</v>
       </c>
       <c r="L567" s="3" t="s">
         <v>50</v>
@@ -76139,13 +76139,13 @@
         <v>65</v>
       </c>
       <c r="Q575" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R575" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S575" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T575" s="3" t="s">
         <v>1207</v>
@@ -76764,13 +76764,13 @@
         <v>196</v>
       </c>
       <c r="Q580" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R580" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S580" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T580" s="3" t="s">
         <v>1207</v>
@@ -77115,13 +77115,13 @@
         <v>1228</v>
       </c>
       <c r="I583" s="3" t="s">
-        <v>1264</v>
+        <v>1258</v>
       </c>
       <c r="J583" s="3" t="s">
-        <v>1265</v>
+        <v>1259</v>
       </c>
       <c r="K583" s="3" t="s">
-        <v>1266</v>
+        <v>1260</v>
       </c>
       <c r="L583" s="3" t="s">
         <v>50</v>
@@ -77264,13 +77264,13 @@
         <v>65</v>
       </c>
       <c r="Q584" s="5">
+        <v>19</v>
+      </c>
+      <c r="R584" s="5">
         <v>18</v>
       </c>
-      <c r="R584" s="5">
-        <v>17</v>
-      </c>
       <c r="S584" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T584" s="3" t="s">
         <v>1207</v>
@@ -77514,13 +77514,13 @@
         <v>140</v>
       </c>
       <c r="Q586" s="5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="R586" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S586" s="5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="T586" s="3" t="s">
         <v>1207</v>
@@ -79139,13 +79139,13 @@
         <v>65</v>
       </c>
       <c r="Q599" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R599" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S599" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T599" s="3" t="s">
         <v>1207</v>
@@ -79389,13 +79389,13 @@
         <v>79</v>
       </c>
       <c r="Q601" s="5">
+        <v>8</v>
+      </c>
+      <c r="R601" s="5">
         <v>7</v>
       </c>
-      <c r="R601" s="5">
-        <v>6</v>
-      </c>
       <c r="S601" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T601" s="3" t="s">
         <v>1207</v>
@@ -80740,13 +80740,13 @@
         <v>45</v>
       </c>
       <c r="I612" s="3" t="s">
-        <v>1258</v>
+        <v>1264</v>
       </c>
       <c r="J612" s="3" t="s">
-        <v>1259</v>
+        <v>1265</v>
       </c>
       <c r="K612" s="3" t="s">
-        <v>1260</v>
+        <v>1266</v>
       </c>
       <c r="L612" s="3" t="s">
         <v>50</v>
@@ -81139,13 +81139,13 @@
         <v>196</v>
       </c>
       <c r="Q615" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R615" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S615" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T615" s="3" t="s">
         <v>1207</v>
@@ -81764,13 +81764,13 @@
         <v>203</v>
       </c>
       <c r="Q620" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R620" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S620" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="T620" s="3" t="s">
         <v>1207</v>
@@ -81990,13 +81990,13 @@
         <v>45</v>
       </c>
       <c r="I622" s="3" t="s">
-        <v>1264</v>
+        <v>1258</v>
       </c>
       <c r="J622" s="3" t="s">
-        <v>1265</v>
+        <v>1259</v>
       </c>
       <c r="K622" s="3" t="s">
-        <v>1266</v>
+        <v>1260</v>
       </c>
       <c r="L622" s="3" t="s">
         <v>50</v>
@@ -82764,13 +82764,13 @@
         <v>203</v>
       </c>
       <c r="Q628" s="5">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R628" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S628" s="5">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="T628" s="3" t="s">
         <v>1207</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 10:58
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -61260,13 +61260,13 @@
         <v>65</v>
       </c>
       <c r="Q457" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R457" s="5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="S457" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T457" s="3" t="s">
         <v>1139</v>
@@ -61510,13 +61510,13 @@
         <v>164</v>
       </c>
       <c r="Q459" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R459" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="S459" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T459" s="3" t="s">
         <v>1139</v>
@@ -63010,13 +63010,13 @@
         <v>164</v>
       </c>
       <c r="Q471" s="5">
+        <v>30</v>
+      </c>
+      <c r="R471" s="5">
         <v>29</v>
       </c>
-      <c r="R471" s="5">
-        <v>28</v>
-      </c>
       <c r="S471" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T471" s="3" t="s">
         <v>1139</v>
@@ -69760,13 +69760,13 @@
         <v>196</v>
       </c>
       <c r="Q525" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R525" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S525" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T525" s="3" t="s">
         <v>1139</v>
@@ -70010,13 +70010,13 @@
         <v>54</v>
       </c>
       <c r="Q527" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R527" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S527" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T527" s="3" t="s">
         <v>1139</v>
@@ -70510,13 +70510,13 @@
         <v>65</v>
       </c>
       <c r="Q531" s="5">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R531" s="5">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S531" s="5">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T531" s="3" t="s">
         <v>1139</v>
@@ -70760,13 +70760,13 @@
         <v>65</v>
       </c>
       <c r="Q533" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="R533" s="5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="S533" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="T533" s="3" t="s">
         <v>1139</v>
@@ -71760,13 +71760,13 @@
         <v>196</v>
       </c>
       <c r="Q541" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R541" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S541" s="5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T541" s="3" t="s">
         <v>1139</v>
@@ -72760,13 +72760,13 @@
         <v>65</v>
       </c>
       <c r="Q549" s="5">
+        <v>35</v>
+      </c>
+      <c r="R549" s="5">
         <v>34</v>
       </c>
-      <c r="R549" s="5">
-        <v>33</v>
-      </c>
       <c r="S549" s="5">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T549" s="3" t="s">
         <v>1139</v>
@@ -76135,13 +76135,13 @@
         <v>196</v>
       </c>
       <c r="Q576" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="R576" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S576" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T576" s="3" t="s">
         <v>1139</v>
@@ -76385,13 +76385,13 @@
         <v>157</v>
       </c>
       <c r="Q578" s="5">
+        <v>16</v>
+      </c>
+      <c r="R578" s="5">
         <v>14</v>
       </c>
-      <c r="R578" s="5">
-        <v>12</v>
-      </c>
       <c r="S578" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="T578" s="3" t="s">
         <v>1139</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 12:33
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -3466,6 +3466,15 @@
     <t xml:space="preserve">108, Đường 4 Đại Học Nông Lâm </t>
   </si>
   <si>
+    <t>2340641</t>
+  </si>
+  <si>
+    <t>Victor</t>
+  </si>
+  <si>
+    <t>89/1/9C, Đường 8</t>
+  </si>
+  <si>
     <t>3057968</t>
   </si>
   <si>
@@ -3473,15 +3482,6 @@
   </si>
   <si>
     <t>71, Đình Phong Phú</t>
-  </si>
-  <si>
-    <t>2340641</t>
-  </si>
-  <si>
-    <t>Victor</t>
-  </si>
-  <si>
-    <t>89/1/9C, Đường 8</t>
   </si>
   <si>
     <t>1-6JP933U</t>
@@ -59165,10 +59165,10 @@
         <v>10</v>
       </c>
       <c r="AA440" s="7">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="AB440" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC440" s="3" t="s">
         <v>1140</v>
@@ -59186,7 +59186,7 @@
         <v>1144</v>
       </c>
       <c r="AH440" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI440" s="3">
         <v>0</v>
@@ -59195,7 +59195,7 @@
         <v>58</v>
       </c>
       <c r="AK440" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
       <c r="AL440" s="3" t="s">
         <v>46</v>
@@ -59207,7 +59207,7 @@
         <v>58</v>
       </c>
       <c r="AO440" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
     </row>
     <row r="441" spans="1:41" x14ac:dyDescent="0.25">
@@ -59236,28 +59236,28 @@
         <v>45</v>
       </c>
       <c r="I441" s="3" t="s">
-        <v>1154</v>
+        <v>233</v>
       </c>
       <c r="J441" s="3" t="s">
-        <v>1155</v>
+        <v>234</v>
       </c>
       <c r="K441" s="3" t="s">
-        <v>1156</v>
+        <v>235</v>
       </c>
       <c r="L441" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M441" s="3" t="s">
-        <v>193</v>
+        <v>154</v>
       </c>
       <c r="N441" s="3" t="s">
-        <v>194</v>
+        <v>155</v>
       </c>
       <c r="O441" s="3" t="s">
-        <v>195</v>
+        <v>156</v>
       </c>
       <c r="P441" s="3" t="s">
-        <v>196</v>
+        <v>157</v>
       </c>
       <c r="Q441" s="3" t="s">
         <v>46</v>
@@ -59290,10 +59290,10 @@
         <v>10</v>
       </c>
       <c r="AA441" s="7">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="AB441" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC441" s="3" t="s">
         <v>1140</v>
@@ -59311,7 +59311,7 @@
         <v>1144</v>
       </c>
       <c r="AH441" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI441" s="3">
         <v>0</v>
@@ -59361,28 +59361,28 @@
         <v>45</v>
       </c>
       <c r="I442" s="3" t="s">
-        <v>233</v>
+        <v>1154</v>
       </c>
       <c r="J442" s="3" t="s">
-        <v>234</v>
+        <v>1155</v>
       </c>
       <c r="K442" s="3" t="s">
-        <v>235</v>
+        <v>1156</v>
       </c>
       <c r="L442" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M442" s="3" t="s">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="N442" s="3" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="O442" s="3" t="s">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="P442" s="3" t="s">
-        <v>157</v>
+        <v>196</v>
       </c>
       <c r="Q442" s="3" t="s">
         <v>46</v>
@@ -59415,7 +59415,7 @@
         <v>10</v>
       </c>
       <c r="AA442" s="7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AB442" s="7">
         <v>1</v>
@@ -59445,7 +59445,7 @@
         <v>58</v>
       </c>
       <c r="AK442" s="6">
-        <v>46301.91933796296</v>
+        <v>46307.90555991898</v>
       </c>
       <c r="AL442" s="3" t="s">
         <v>46</v>
@@ -59457,7 +59457,7 @@
         <v>58</v>
       </c>
       <c r="AO442" s="6">
-        <v>46301.91933796296</v>
+        <v>46307.90555991898</v>
       </c>
     </row>
     <row r="443" spans="1:41" x14ac:dyDescent="0.25">
@@ -59760,13 +59760,13 @@
         <v>65</v>
       </c>
       <c r="Q445" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R445" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S445" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T445" s="3" t="s">
         <v>1139</v>
@@ -69385,13 +69385,13 @@
         <v>65</v>
       </c>
       <c r="Q522" s="5">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R522" s="5">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S522" s="5">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T522" s="3" t="s">
         <v>1139</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 13:30
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -3466,6 +3466,15 @@
     <t xml:space="preserve">108, Đường 4 Đại Học Nông Lâm </t>
   </si>
   <si>
+    <t>3057968</t>
+  </si>
+  <si>
+    <t>Anh Hùng ( Trái Cây )</t>
+  </si>
+  <si>
+    <t>71, Đình Phong Phú</t>
+  </si>
+  <si>
     <t>2340641</t>
   </si>
   <si>
@@ -3473,15 +3482,6 @@
   </si>
   <si>
     <t>89/1/9C, Đường 8</t>
-  </si>
-  <si>
-    <t>3057968</t>
-  </si>
-  <si>
-    <t>Anh Hùng ( Trái Cây )</t>
-  </si>
-  <si>
-    <t>71, Đình Phong Phú</t>
   </si>
   <si>
     <t>1-6JP933U</t>
@@ -59165,10 +59165,10 @@
         <v>10</v>
       </c>
       <c r="AA440" s="7">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="AB440" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC440" s="3" t="s">
         <v>1140</v>
@@ -59186,7 +59186,7 @@
         <v>1144</v>
       </c>
       <c r="AH440" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI440" s="3">
         <v>0</v>
@@ -59195,7 +59195,7 @@
         <v>58</v>
       </c>
       <c r="AK440" s="6">
-        <v>46301.91933796296</v>
+        <v>46307.90555991898</v>
       </c>
       <c r="AL440" s="3" t="s">
         <v>46</v>
@@ -59207,7 +59207,7 @@
         <v>58</v>
       </c>
       <c r="AO440" s="6">
-        <v>46301.91933796296</v>
+        <v>46307.90555991898</v>
       </c>
     </row>
     <row r="441" spans="1:41" x14ac:dyDescent="0.25">
@@ -59236,28 +59236,28 @@
         <v>45</v>
       </c>
       <c r="I441" s="3" t="s">
-        <v>233</v>
+        <v>1154</v>
       </c>
       <c r="J441" s="3" t="s">
-        <v>234</v>
+        <v>1155</v>
       </c>
       <c r="K441" s="3" t="s">
-        <v>235</v>
+        <v>1156</v>
       </c>
       <c r="L441" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M441" s="3" t="s">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="N441" s="3" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="O441" s="3" t="s">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="P441" s="3" t="s">
-        <v>157</v>
+        <v>196</v>
       </c>
       <c r="Q441" s="3" t="s">
         <v>46</v>
@@ -59290,10 +59290,10 @@
         <v>10</v>
       </c>
       <c r="AA441" s="7">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="AB441" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC441" s="3" t="s">
         <v>1140</v>
@@ -59311,7 +59311,7 @@
         <v>1144</v>
       </c>
       <c r="AH441" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI441" s="3">
         <v>0</v>
@@ -59361,28 +59361,28 @@
         <v>45</v>
       </c>
       <c r="I442" s="3" t="s">
-        <v>1154</v>
+        <v>233</v>
       </c>
       <c r="J442" s="3" t="s">
-        <v>1155</v>
+        <v>234</v>
       </c>
       <c r="K442" s="3" t="s">
-        <v>1156</v>
+        <v>235</v>
       </c>
       <c r="L442" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M442" s="3" t="s">
-        <v>193</v>
+        <v>154</v>
       </c>
       <c r="N442" s="3" t="s">
-        <v>194</v>
+        <v>155</v>
       </c>
       <c r="O442" s="3" t="s">
-        <v>195</v>
+        <v>156</v>
       </c>
       <c r="P442" s="3" t="s">
-        <v>196</v>
+        <v>157</v>
       </c>
       <c r="Q442" s="3" t="s">
         <v>46</v>
@@ -59415,7 +59415,7 @@
         <v>10</v>
       </c>
       <c r="AA442" s="7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AB442" s="7">
         <v>1</v>
@@ -59445,7 +59445,7 @@
         <v>58</v>
       </c>
       <c r="AK442" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
       <c r="AL442" s="3" t="s">
         <v>46</v>
@@ -59457,7 +59457,7 @@
         <v>58</v>
       </c>
       <c r="AO442" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
     </row>
     <row r="443" spans="1:41" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 16:45
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -77635,13 +77635,13 @@
         <v>79</v>
       </c>
       <c r="Q588" s="5">
+        <v>30</v>
+      </c>
+      <c r="R588" s="5">
         <v>29</v>
       </c>
-      <c r="R588" s="5">
-        <v>28</v>
-      </c>
       <c r="S588" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T588" s="3" t="s">
         <v>1139</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 18:30
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -60885,13 +60885,13 @@
         <v>65</v>
       </c>
       <c r="Q454" s="5">
+        <v>21</v>
+      </c>
+      <c r="R454" s="5">
         <v>20</v>
       </c>
-      <c r="R454" s="5">
-        <v>19</v>
-      </c>
       <c r="S454" s="5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="T454" s="3" t="s">
         <v>1139</v>
@@ -72260,13 +72260,13 @@
         <v>65</v>
       </c>
       <c r="Q545" s="5">
+        <v>20</v>
+      </c>
+      <c r="R545" s="5">
         <v>19</v>
       </c>
-      <c r="R545" s="5">
-        <v>18</v>
-      </c>
       <c r="S545" s="5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="T545" s="3" t="s">
         <v>1139</v>

</xml_diff>